<commit_message>
downloader working, create excel sheet to know status codes for archive links
</commit_message>
<xml_diff>
--- a/reports/processed/hamzasiyam.com_snapshots.xlsx
+++ b/reports/processed/hamzasiyam.com_snapshots.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Snapshots" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Snapshots_HTTP" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1014,6 +1015,588 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="58" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Capture</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Capture Link</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Month Day, Year</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Hour, Minute, Second AM/PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>http://web.archive.org/web/20230122175639/hamzasiyam.com</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>January 22, 2023</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>05:56:39 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>http://web.archive.org/web/20230318090601/hamzasiyam.com</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>March 18, 2023</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>09:06:01 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>http://web.archive.org/web/20230318090603/hamzasiyam.com</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>March 18, 2023</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>09:06:03 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>http://web.archive.org/web/20230321195243/hamzasiyam.com</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>March 21, 2023</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>07:52:43 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>http://web.archive.org/web/20230322144033/hamzasiyam.com</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>March 22, 2023</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>02:40:33 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>http://web.archive.org/web/20230330025053/hamzasiyam.com</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>March 30, 2023</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>02:50:53 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>http://web.archive.org/web/20230417043730/hamzasiyam.com</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>April 17, 2023</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>04:37:30 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>http://web.archive.org/web/20230417043731/hamzasiyam.com</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>April 17, 2023</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>04:37:31 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>http://web.archive.org/web/20230610133247/hamzasiyam.com</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>June 10, 2023</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>01:32:47 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>http://web.archive.org/web/20230704174118/hamzasiyam.com</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>July 04, 2023</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>05:41:18 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>http://web.archive.org/web/20230704174120/hamzasiyam.com</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>July 04, 2023</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>05:41:20 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>http://web.archive.org/web/20230902212516/hamzasiyam.com</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>September 02, 2023</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>09:25:16 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>http://web.archive.org/web/20230902212517/hamzasiyam.com</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>September 02, 2023</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>09:25:17 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>http://web.archive.org/web/20230929160346/hamzasiyam.com</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>September 29, 2023</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>04:03:46 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>http://web.archive.org/web/20231111032616/hamzasiyam.com</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>November 11, 2023</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>03:26:16 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>http://web.archive.org/web/20231111032617/hamzasiyam.com</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>November 11, 2023</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>03:26:17 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>http://web.archive.org/web/20231208062316/hamzasiyam.com</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>December 08, 2023</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>06:23:16 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>http://web.archive.org/web/20231209140527/hamzasiyam.com</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>December 09, 2023</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>02:05:27 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>http://web.archive.org/web/20231225174341/hamzasiyam.com</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>December 25, 2023</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>05:43:41 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>http://web.archive.org/web/20240131112905/hamzasiyam.com</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>January 31, 2024</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>11:29:05 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>http://web.archive.org/web/20240209174537/hamzasiyam.com</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>February 09, 2024</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>05:45:37 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>http://web.archive.org/web/20240216041901/hamzasiyam.com</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>February 16, 2024</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>04:19:01 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>http://web.archive.org/web/20240228083023/hamzasiyam.com</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>February 28, 2024</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>08:30:23 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>http://web.archive.org/web/20240315091539/hamzasiyam.com</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>March 15, 2024</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>09:15:39 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>http://web.archive.org/web/20240414063446/hamzasiyam.com</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>April 14, 2024</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>06:34:46 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>http://web.archive.org/web/20240514081319/hamzasiyam.com</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>May 14, 2024</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>08:13:19 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>http://web.archive.org/web/20240613063610/hamzasiyam.com</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>June 13, 2024</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>06:36:10 AM</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
summaries added to program
</commit_message>
<xml_diff>
--- a/reports/processed/hamzasiyam.com_snapshots.xlsx
+++ b/reports/processed/hamzasiyam.com_snapshots.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1001,6 +1001,26 @@
       <c r="D28" s="3" t="inlineStr">
         <is>
           <t>06:36:10 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>https://web.archive.org/web/20240807201133/hamzasiyam.com</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>August 07, 2024</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>08:11:33 PM</t>
         </is>
       </c>
     </row>
@@ -1015,7 +1035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1583,6 +1603,26 @@
       <c r="D28" s="3" t="inlineStr">
         <is>
           <t>06:36:10 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>http://web.archive.org/web/20240807201133/hamzasiyam.com</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>August 07, 2024</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>08:11:33 PM</t>
         </is>
       </c>
     </row>
@@ -1602,7 +1642,7 @@
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="29" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1624,7 +1664,7 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
@@ -1633,7 +1673,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>June 13, 2024 06:36:10 AM</t>
+          <t>August 07, 2024 08:11:33 PM</t>
         </is>
       </c>
     </row>

</xml_diff>